<commit_message>
links to those bought
</commit_message>
<xml_diff>
--- a/hardware/doc/BOM.xlsx
+++ b/hardware/doc/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Katarzyna\Documents\PROJECTS\NI-watch\hardware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8086E2-1D17-47A1-9A82-6BB5A0FD398B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A854FD80-5EF9-4F1C-9348-B8BC25A4D579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="78">
   <si>
     <t>Reference</t>
   </si>
@@ -184,13 +184,100 @@
   </si>
   <si>
     <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
+  </si>
+  <si>
+    <t>MC34063ADR</t>
+  </si>
+  <si>
+    <t>ic conv dc-dc Ti</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/mc34063adr/regulatory-napiecia-uklady-dc-dc/texas-instruments/</t>
+  </si>
+  <si>
+    <t>SD8328-101-R</t>
+  </si>
+  <si>
+    <t>L 100uH smd 800mA</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/sd8328-101-r/dlawiki-smd-mocy/eaton-electronics/</t>
+  </si>
+  <si>
+    <t>IRF740PBF</t>
+  </si>
+  <si>
+    <t>tranzystor</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/irf740pbf/tranzystory-z-kanalem-n-tht/vishay/</t>
+  </si>
+  <si>
+    <t>rezysotry</t>
+  </si>
+  <si>
+    <t>https://sklep.avt.pl/pl/products/zestaw-rezystorow-smd-0805-800-sztuk-avt701-805-167603.html?query_id=5</t>
+  </si>
+  <si>
+    <t>zestaw kondensatorów</t>
+  </si>
+  <si>
+    <t>https://sklep.avt.pl/pl/products/zestaw-kondensatorow-smd-1206-120-sztuk-avt714-169129.html?query_id=6</t>
+  </si>
+  <si>
+    <t>nucleo-f091rc</t>
+  </si>
+  <si>
+    <t>MCU</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/nucleo-f091rc/zestawy-do-ukladow-stm/stmicroelectronics/</t>
+  </si>
+  <si>
+    <t>100uF 16v</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/km100_16/kondensatory-elektrolityczne-tht/samxon/km-100u-16v/</t>
+  </si>
+  <si>
+    <t>LM78L05</t>
+  </si>
+  <si>
+    <t>STABILIZATOR</t>
+  </si>
+  <si>
+    <t>UF4007</t>
+  </si>
+  <si>
+    <t>Dioda: prostownicza; THT; 1kV; 1A; Ammo Pack; Ifsm: 30A; DO41; Ir: 5uA</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/uf4007-dio/diody-uniwersalne-tht/diotec-semiconductor/uf4007/</t>
+  </si>
+  <si>
+    <t>MPEM-4U7R27.5/250</t>
+  </si>
+  <si>
+    <t>4u7/250V</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/mpem-4u7r27.5_250/kondensatory-foliowe-tht/sr-passives/</t>
+  </si>
+  <si>
+    <t>CS1206-0.22R-1%</t>
+  </si>
+  <si>
+    <t>thick film</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/cs1206-0.22r-1%25/rezystory-smd/royal-ohm/cs06w4f220lt5e/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,16 +293,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF9900"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2E353B"/>
+      <name val="Lato"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA9999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -223,14 +335,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperłącze" xfId="1" builtinId="8"/>
@@ -558,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F8717B9-DC92-4B11-8F46-F871C13CDF09}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
@@ -869,13 +1017,137 @@
         <v>10</v>
       </c>
     </row>
+    <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="17" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="4"/>
+      <c r="C21" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" ht="53" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C5" r:id="rId1" xr:uid="{1A42116A-1EF3-4048-A4BD-E4ED4A7D02BE}"/>
+    <hyperlink ref="C17" r:id="rId2" xr:uid="{8581EEE7-E374-4A56-8804-1A47736BE76F}"/>
+    <hyperlink ref="C18" r:id="rId3" xr:uid="{BD4AFEA6-13D7-4950-9BE6-2341F9423F72}"/>
+    <hyperlink ref="C19" r:id="rId4" xr:uid="{9778816E-08E1-4F2B-810E-67ADD6376E06}"/>
+    <hyperlink ref="C20" r:id="rId5" xr:uid="{5DB19C3D-3083-4E03-BD98-101BFB408342}"/>
+    <hyperlink ref="C21" r:id="rId6" xr:uid="{AC9D2F71-025E-4B31-BFC6-0807E766D54B}"/>
+    <hyperlink ref="C22" r:id="rId7" xr:uid="{ACD16ED1-B94F-40F2-8064-6F873D901AD1}"/>
+    <hyperlink ref="C23" r:id="rId8" xr:uid="{380D16AD-66EF-4FE1-9C41-09964C9E3386}"/>
+    <hyperlink ref="C25" r:id="rId9" xr:uid="{47C38A91-5DCF-4B4D-9FBF-0C343D530894}"/>
+    <hyperlink ref="C26" r:id="rId10" xr:uid="{5D59F146-F4F6-4542-8E0D-EAB945DA3C29}"/>
+    <hyperlink ref="C27" r:id="rId11" xr:uid="{BFE93090-5044-4DAF-8837-507FE5BB347F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
full BOM, mounted - verified footprints ok (- radiator hole)
</commit_message>
<xml_diff>
--- a/hardware/doc/BOM.xlsx
+++ b/hardware/doc/BOM.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Katarzyna\Documents\PROJECTS\NI-watch\hardware\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A854FD80-5EF9-4F1C-9348-B8BC25A4D579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5F74DA-C27D-4C23-BF97-526DEA85E869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-36" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="zegarek" sheetId="2" r:id="rId1"/>
     <sheet name="Arkusz1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">zegarek!$A$1:$F$15</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">zegarek!$A$1:$F$33</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="67">
   <si>
     <t>Reference</t>
   </si>
@@ -81,9 +81,6 @@
     <t>C3</t>
   </si>
   <si>
-    <t>4u7 250V</t>
-  </si>
-  <si>
     <t>Capacitor_THT:CP_Axial_L25.0mm_D10.0mm_P30.00mm_Horizontal</t>
   </si>
   <si>
@@ -93,9 +90,6 @@
     <t>UF5400</t>
   </si>
   <si>
-    <t>http://www.vishay.com/docs/88756/uf5400.pdf</t>
-  </si>
-  <si>
     <t>Diode_THT:D_DO-201AD_P15.24mm_Horizontal</t>
   </si>
   <si>
@@ -111,36 +105,21 @@
     <t>J2</t>
   </si>
   <si>
-    <t>Conn_01x02_Pin</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
-    <t>100uH</t>
-  </si>
-  <si>
     <t>Inductor_SMD:L_10.4x10.4_H4.8</t>
   </si>
   <si>
     <t>Q1</t>
   </si>
   <si>
-    <t>IRF740</t>
-  </si>
-  <si>
-    <t>http://www.vishay.com/docs/91054/91054.pdf</t>
-  </si>
-  <si>
     <t>Package_TO_SOT_THT:TO-220-3_Vertical</t>
   </si>
   <si>
     <t>R1</t>
   </si>
   <si>
-    <t>0R22</t>
-  </si>
-  <si>
     <t>Resistor_SMD:R_1206_3216Metric_Pad1.30x1.75mm_HandSolder</t>
   </si>
   <si>
@@ -177,107 +156,95 @@
     <t>U1</t>
   </si>
   <si>
-    <t>MC34063AD</t>
-  </si>
-  <si>
-    <t>http://www.onsemi.com/pub_link/Collateral/MC34063A-D.PDF</t>
-  </si>
-  <si>
     <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
   </si>
   <si>
     <t>MC34063ADR</t>
   </si>
   <si>
-    <t>ic conv dc-dc Ti</t>
-  </si>
-  <si>
     <t>https://www.tme.eu/pl/details/mc34063adr/regulatory-napiecia-uklady-dc-dc/texas-instruments/</t>
   </si>
   <si>
-    <t>SD8328-101-R</t>
-  </si>
-  <si>
-    <t>L 100uH smd 800mA</t>
-  </si>
-  <si>
     <t>https://www.tme.eu/pl/details/sd8328-101-r/dlawiki-smd-mocy/eaton-electronics/</t>
   </si>
   <si>
     <t>IRF740PBF</t>
   </si>
   <si>
-    <t>tranzystor</t>
-  </si>
-  <si>
     <t>https://www.tme.eu/pl/details/irf740pbf/tranzystory-z-kanalem-n-tht/vishay/</t>
   </si>
   <si>
-    <t>rezysotry</t>
-  </si>
-  <si>
-    <t>https://sklep.avt.pl/pl/products/zestaw-rezystorow-smd-0805-800-sztuk-avt701-805-167603.html?query_id=5</t>
-  </si>
-  <si>
-    <t>zestaw kondensatorów</t>
-  </si>
-  <si>
-    <t>https://sklep.avt.pl/pl/products/zestaw-kondensatorow-smd-1206-120-sztuk-avt714-169129.html?query_id=6</t>
-  </si>
-  <si>
-    <t>nucleo-f091rc</t>
-  </si>
-  <si>
-    <t>MCU</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/pl/details/nucleo-f091rc/zestawy-do-ukladow-stm/stmicroelectronics/</t>
-  </si>
-  <si>
-    <t>100uF 16v</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/pl/details/km100_16/kondensatory-elektrolityczne-tht/samxon/km-100u-16v/</t>
-  </si>
-  <si>
-    <t>LM78L05</t>
-  </si>
-  <si>
-    <t>STABILIZATOR</t>
-  </si>
-  <si>
-    <t>UF4007</t>
-  </si>
-  <si>
-    <t>Dioda: prostownicza; THT; 1kV; 1A; Ammo Pack; Ifsm: 30A; DO41; Ir: 5uA</t>
-  </si>
-  <si>
     <t>https://www.tme.eu/pl/details/uf4007-dio/diody-uniwersalne-tht/diotec-semiconductor/uf4007/</t>
   </si>
   <si>
-    <t>MPEM-4U7R27.5/250</t>
-  </si>
-  <si>
-    <t>4u7/250V</t>
-  </si>
-  <si>
     <t>https://www.tme.eu/pl/details/mpem-4u7r27.5_250/kondensatory-foliowe-tht/sr-passives/</t>
   </si>
   <si>
-    <t>CS1206-0.22R-1%</t>
-  </si>
-  <si>
-    <t>thick film</t>
-  </si>
-  <si>
     <t>https://www.tme.eu/pl/details/cs1206-0.22r-1%25/rezystory-smd/royal-ohm/cs06w4f220lt5e/</t>
+  </si>
+  <si>
+    <t>100uH smd 800mA SD8328-101-R</t>
+  </si>
+  <si>
+    <t>4u7 250V MPEM-4U7R27.5/250</t>
+  </si>
+  <si>
+    <t>0R22 thic film prec.</t>
+  </si>
+  <si>
+    <t>PÓŁPRZEWODNIKI</t>
+  </si>
+  <si>
+    <t>KONEKTORY</t>
+  </si>
+  <si>
+    <t>INDUKCYJNE</t>
+  </si>
+  <si>
+    <t>UKŁADY SCALONE</t>
+  </si>
+  <si>
+    <t>REZYSTORY</t>
+  </si>
+  <si>
+    <t>POJEMNOŚCI</t>
+  </si>
+  <si>
+    <t>OK.</t>
+  </si>
+  <si>
+    <t>MECHANICZNE</t>
+  </si>
+  <si>
+    <t>kołek na banan</t>
+  </si>
+  <si>
+    <t>śrubka M3</t>
+  </si>
+  <si>
+    <t>radiator M3</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/ua17-to220/radiatory/fischer-elektronik/sk13-35-al-220/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/pl/details/fix-mae-15tv/kolki-montazowe-plastikowe/fix-fasten/</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>ZAMÓWIONE</t>
+  </si>
+  <si>
+    <t>dystans m3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -294,40 +261,38 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="238"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFF9900"/>
-      <name val="Arial"/>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <charset val="238"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF2E353B"/>
       <name val="Lato"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEA9999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -335,48 +300,48 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -387,6 +352,7 @@
   <dxfs count="5">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -429,15 +395,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE45E825-427A-4216-9E8C-3B0CB1A5CE96}" name="zegarek" displayName="zegarek" ref="A1:F15" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:F15" xr:uid="{BE45E825-427A-4216-9E8C-3B0CB1A5CE96}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE45E825-427A-4216-9E8C-3B0CB1A5CE96}" name="zegarek" displayName="zegarek" ref="A1:F33" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:F33" xr:uid="{BE45E825-427A-4216-9E8C-3B0CB1A5CE96}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C3D99145-EA13-40C9-B186-FAE62FD011E7}" uniqueName="1" name="Reference" queryTableFieldId="1" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{47C4836D-357E-4AA9-98D4-A1397AE59728}" uniqueName="2" name="Value" queryTableFieldId="2" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{4F34AC66-3A1C-4FC4-8251-1F74595D2C66}" uniqueName="3" name="Datasheet" queryTableFieldId="3" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{5B3B7FB8-4136-4759-B41F-33DCBFA1A37A}" uniqueName="4" name="Footprint" queryTableFieldId="4" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{C3D99145-EA13-40C9-B186-FAE62FD011E7}" uniqueName="1" name="Reference" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{47C4836D-357E-4AA9-98D4-A1397AE59728}" uniqueName="2" name="Value" queryTableFieldId="2" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{4F34AC66-3A1C-4FC4-8251-1F74595D2C66}" uniqueName="3" name="Datasheet" queryTableFieldId="3" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{5B3B7FB8-4136-4759-B41F-33DCBFA1A37A}" uniqueName="4" name="Footprint" queryTableFieldId="4" dataDxfId="4"/>
     <tableColumn id="5" xr3:uid="{B58912A5-DF1D-47C0-96B2-61F9C0E5C3FC}" uniqueName="5" name="Qty" queryTableFieldId="5"/>
-    <tableColumn id="6" xr3:uid="{AEFBD6C0-8C0A-4BC4-A830-B6EE33F7C20D}" uniqueName="6" name="DNP" queryTableFieldId="6" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{AEFBD6C0-8C0A-4BC4-A830-B6EE33F7C20D}" uniqueName="6" name="DNP" queryTableFieldId="6" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -706,7 +672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F8717B9-DC92-4B11-8F46-F871C13CDF09}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
@@ -738,237 +704,165 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
+      <c r="A2" s="7"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="F2" s="7"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
+      <c r="A3" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="11"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
+        <v>6</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>7</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
+        <v>13</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
-        <v>10</v>
-      </c>
+      <c r="A7" s="7"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="7"/>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>10</v>
-      </c>
+      <c r="A8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="7"/>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" t="s">
-        <v>30</v>
+        <v>15</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
+        <v>24</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s">
-        <v>10</v>
-      </c>
+      <c r="A11" s="7"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12" t="s">
-        <v>10</v>
-      </c>
+      <c r="A12" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="7"/>
+      <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" t="s">
-        <v>42</v>
+        <v>18</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -979,16 +873,16 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" t="s">
-        <v>44</v>
+        <v>21</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -998,156 +892,313 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="A15" s="7"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B18" s="12"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D15" t="s">
-        <v>48</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="17" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="3" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" t="s">
+        <v>33</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="7"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="F25" s="7"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="7" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B26" s="11"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="F26" s="7"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="4" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="7"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="7"/>
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="5" t="s">
+      <c r="B29" s="13"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="7"/>
+      <c r="F29" s="7"/>
+    </row>
+    <row r="30" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="B30" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="7"/>
+      <c r="E30">
+        <v>4</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B31" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="4" t="s">
+      <c r="C31" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31">
+        <v>4</v>
+      </c>
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="7"/>
+      <c r="B32" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="5" t="s">
+      <c r="C32" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="7"/>
+      <c r="E32">
+        <v>5</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="7"/>
+      <c r="B33" s="9" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
+      <c r="C33" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" ht="53" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>77</v>
-      </c>
+      <c r="D33" s="7"/>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="5"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="5"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+    </row>
+    <row r="38" spans="1:6" ht="15.5" x14ac:dyDescent="0.45">
+      <c r="A38" s="3"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="4"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="4"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C5" r:id="rId1" xr:uid="{1A42116A-1EF3-4048-A4BD-E4ED4A7D02BE}"/>
-    <hyperlink ref="C17" r:id="rId2" xr:uid="{8581EEE7-E374-4A56-8804-1A47736BE76F}"/>
-    <hyperlink ref="C18" r:id="rId3" xr:uid="{BD4AFEA6-13D7-4950-9BE6-2341F9423F72}"/>
-    <hyperlink ref="C19" r:id="rId4" xr:uid="{9778816E-08E1-4F2B-810E-67ADD6376E06}"/>
-    <hyperlink ref="C20" r:id="rId5" xr:uid="{5DB19C3D-3083-4E03-BD98-101BFB408342}"/>
-    <hyperlink ref="C21" r:id="rId6" xr:uid="{AC9D2F71-025E-4B31-BFC6-0807E766D54B}"/>
-    <hyperlink ref="C22" r:id="rId7" xr:uid="{ACD16ED1-B94F-40F2-8064-6F873D901AD1}"/>
-    <hyperlink ref="C23" r:id="rId8" xr:uid="{380D16AD-66EF-4FE1-9C41-09964C9E3386}"/>
-    <hyperlink ref="C25" r:id="rId9" xr:uid="{47C38A91-5DCF-4B4D-9FBF-0C343D530894}"/>
-    <hyperlink ref="C26" r:id="rId10" xr:uid="{5D59F146-F4F6-4542-8E0D-EAB945DA3C29}"/>
-    <hyperlink ref="C27" r:id="rId11" xr:uid="{BFE93090-5044-4DAF-8837-507FE5BB347F}"/>
+    <hyperlink ref="C27" r:id="rId1" xr:uid="{2D89C628-A252-41DD-8026-21E65DE54623}"/>
+    <hyperlink ref="C10" r:id="rId2" xr:uid="{1A2B394C-ABDE-4A3F-A0C1-13AE3EFEFDB7}"/>
+    <hyperlink ref="C17" r:id="rId3" xr:uid="{1CEEEE57-C3DF-499C-98D5-02919618F2E2}"/>
+    <hyperlink ref="C6" r:id="rId4" xr:uid="{78CFBF14-4062-41B8-8CC4-6803FE94AB0B}"/>
+    <hyperlink ref="C9" r:id="rId5" xr:uid="{ADCB10DF-46C5-4A1F-BB07-1C6C6C8A6094}"/>
+    <hyperlink ref="C20" r:id="rId6" xr:uid="{5915D1B4-F833-4E21-B396-1EB88969B5D3}"/>
+    <hyperlink ref="C30" r:id="rId7" xr:uid="{14BEEBAD-5904-4AF4-9E8E-4E0C3459533A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId12"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>